<commit_message>
New files and tasks added
</commit_message>
<xml_diff>
--- a/SDET_PW/test-data/loan.xlsx
+++ b/SDET_PW/test-data/loan.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="19080" windowHeight="4320" activeTab="1"/>
+    <workbookView windowWidth="19080" windowHeight="5535" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -69,7 +69,7 @@
     <t>Validity</t>
   </si>
   <si>
-    <t>Aswin</t>
+    <t>A</t>
   </si>
   <si>
     <t>aaa@email.com</t>
@@ -1347,7 +1347,7 @@
         <v>9999999999</v>
       </c>
       <c r="D2" t="s">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="3" spans="1:4">

</xml_diff>